<commit_message>
feat: 模板生成器 6→5 卡 — weights/guide/PERSON_RANGE/SEED_TASKS 更新，重新生成 物流团队绩效V1.xlsx
</commit_message>
<xml_diff>
--- a/物流团队绩效/物流团队绩效V1.xlsx
+++ b/物流团队绩效/物流团队绩效V1.xlsx
@@ -660,7 +660,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>绿≥85 / 黄70-84.9 / 红&lt;70 / NA灰；实习生（张雨洁）算分但不排名不挂钱</t>
+          <t>绿≥85 / 黄70-84.9 / 红&lt;70 / NA灰；其他项（机动支援）不设卡，只任务块月度考核</t>
         </is>
       </c>
     </row>
@@ -675,12 +675,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>V1</t>
+          <t>V1.1</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-08-19 定稿；权重固定，2027-02 复盘</t>
+          <t>2026-08-26 定稿：卡结构 6→5（雨洁卡撤销，K23/K24/K25 并入郑舒漫并重新配权）；权重固定，2027-02 复盘</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -779,12 +779,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>头程FOB</t>
+          <t>FOB · 特殊发运 · 进口 · 单据（接雨洁）</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>FOB(单证15+订舱10) · FCA执行25 · 请款20</t>
+          <t>FOB(单证7.5+订舱5) · FCA执行12.5 · 请款10 · 特殊发运20 · 进口时效10 · 账单协同5</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -869,33 +869,6 @@
         </is>
       </c>
       <c r="E8" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>张雨洁</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>物流实习生</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>样机发运、进口、账单核对</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>特殊发运40 · 进口时效20 · 账单协同10（不排名不挂钱）</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
         <is>
           <t>30</t>
         </is>
@@ -1323,7 +1296,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>15</v>
+        <v>7.5</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -1373,7 +1346,7 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -1423,7 +1396,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>25</v>
+        <v>12.5</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -1469,7 +1442,7 @@
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -1490,70 +1463,67 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>K11</t>
+          <t>K23</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>黄婷</t>
+          <t>郑舒漫</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>B端中转</t>
+          <t>特殊发运</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>成本</t>
+          <t>时效</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>成本-计算</t>
-        </is>
-      </c>
-      <c r="F14" t="n">
-        <v>15</v>
+          <t>达标率</t>
+        </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>欧/台</t>
+          <t>%</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>签收数量A / 运费折欧B</t>
+          <t>达标单数 / 总单数</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>当月核对账单</t>
+          <t>头程大表；长期易仓</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>当月签收</t>
+          <t>当月签收，按运输方式分段</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>K12</t>
+          <t>K24</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>黄婷</t>
+          <t>郑舒漫</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>B端中转</t>
+          <t>进口业务</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1572,7 +1542,7 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -1581,72 +1551,65 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>签收单+分段标准</t>
+          <t>待定</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>DE1/DK2/AT2/SE1/SI2工作日；旺3-6淡7-2</t>
+          <t>分段标准8月底前定，否则首月NA</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>K13</t>
+          <t>K25</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>黄婷</t>
+          <t>郑舒漫</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>目的国计划</t>
+          <t>财务</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>缺货率</t>
+          <t>账单协同-请款</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>上限</t>
-        </is>
-      </c>
-      <c r="F16" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
+          <t>请款</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
         <v>5</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>实际缺货率(小数)</t>
+          <t>迟报工作日数 / 请款金额占比(小数)</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>在库+待发+在途表</t>
+          <t>请款记录</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>每周一交付计划</t>
+          <t>账单协同表</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>K14</t>
+          <t>K11</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1656,50 +1619,50 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>目的国计划</t>
+          <t>B端中转</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>缺货时间</t>
+          <t>成本</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>上限</t>
+          <t>成本-计算</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>天</t>
+          <t>欧/台</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>实际缺货天数</t>
+          <t>签收数量A / 运费折欧B</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>在库+待发+在途表</t>
+          <t>当月核对账单</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>缺货持续≤7天</t>
+          <t>当月签收</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>K15</t>
+          <t>K12</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1709,43 +1672,47 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>B端库存</t>
+          <t>B端中转</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>时效</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>库存综合</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr"/>
+          <t>达标率</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
       <c r="H18" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>长周期占比(小数) / 平均库龄(天) / 单台库内成本(欧)</t>
+          <t>达标单数 / 总单数</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>各仓库存表+账单</t>
+          <t>签收单+分段标准</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>≤3%/≤120天/≤5欧</t>
+          <t>DE1/DK2/AT2/SE1/SI2工作日；旺3-6淡7-2</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>K16</t>
+          <t>K13</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1755,43 +1722,50 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>财务</t>
+          <t>目的国计划</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>请款-B端仓库内</t>
+          <t>缺货率</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>请款</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr"/>
+          <t>上限</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
       <c r="H19" t="n">
-        <v>7.5</v>
+        <v>5</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>迟报工作日数 / 请款金额占比(小数)</t>
+          <t>实际缺货率(小数)</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>请款记录</t>
+          <t>在库+待发+在途表</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>10号前，≥90%</t>
+          <t>每周一交付计划</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>K17</t>
+          <t>K14</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1801,199 +1775,188 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>财务</t>
+          <t>目的国计划</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>请款-海外仓调拨</t>
+          <t>缺货时间</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>请款</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr"/>
+          <t>上限</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>7</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>天</t>
+        </is>
+      </c>
       <c r="H20" t="n">
-        <v>7.5</v>
+        <v>5</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>迟报工作日数 / 请款金额占比(小数)</t>
+          <t>实际缺货天数</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>请款记录</t>
+          <t>在库+待发+在途表</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>10号前，≥90%</t>
+          <t>缺货持续≤7天</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>K18</t>
+          <t>K15</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>吴定佳</t>
+          <t>黄婷</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>一件代发</t>
+          <t>B端库存</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>成本</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>成本-计算</t>
-        </is>
-      </c>
-      <c r="F21" t="n">
-        <v>15</v>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>欧/台</t>
-        </is>
-      </c>
+          <t>库存综合</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>出库数量A / 运费折欧B</t>
+          <t>长周期占比(小数) / 平均库龄(天) / 单台库内成本(欧)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>正向仓账单+领星/易仓</t>
+          <t>各仓库存表+账单</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>当月出库</t>
+          <t>≤3%/≤120天/≤5欧</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>K19</t>
+          <t>K16</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>吴定佳</t>
+          <t>黄婷</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>一件代发</t>
+          <t>财务</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>时效</t>
+          <t>请款-B端仓库内</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>达标率</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
+          <t>请款</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>16</v>
+        <v>7.5</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>达标单数 / 总单数</t>
+          <t>迟报工作日数 / 请款金额占比(小数)</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>渠道承诺时效</t>
+          <t>请款记录</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>出库单生成→签收；分段标准任务块定稿</t>
+          <t>10号前，≥90%</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>K20</t>
+          <t>K17</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>吴定佳</t>
+          <t>黄婷</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>售后物流</t>
+          <t>财务</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>退件率</t>
+          <t>请款-海外仓调拨</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>上限</t>
-        </is>
-      </c>
-      <c r="F23" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
+          <t>请款</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>物流因素退件率(小数)</t>
+          <t>迟报工作日数 / 请款金额占比(小数)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>客服数据</t>
+          <t>请款记录</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>≤2%</t>
+          <t>10号前，≥90%</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>K21</t>
+          <t>K18</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2003,43 +1966,50 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>C端库存</t>
+          <t>一件代发</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>成本</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>库存综合</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr"/>
+          <t>成本-计算</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>15</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>欧/台</t>
+        </is>
+      </c>
       <c r="H24" t="n">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>长周期占比(小数) / 平均库龄(天) / 单台库内成本(欧)</t>
+          <t>出库数量A / 运费折欧B</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>各仓库存表+账单</t>
+          <t>正向仓账单+领星/易仓</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>≤3%/≤120天/≤5欧</t>
+          <t>当月出库</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>K22</t>
+          <t>K19</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2049,64 +2019,71 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>财务</t>
+          <t>一件代发</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>请款-C端仓库内</t>
+          <t>时效</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>请款</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr"/>
+          <t>达标率</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
       <c r="H25" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>迟报工作日数 / 请款金额占比(小数)</t>
+          <t>达标单数 / 总单数</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>请款记录</t>
+          <t>渠道承诺时效</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>10号前，≥90%</t>
+          <t>出库单生成→签收；分段标准任务块定稿</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>K23</t>
+          <t>K20</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>张雨洁</t>
+          <t>吴定佳</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>特殊发运</t>
+          <t>售后物流</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>时效</t>
+          <t>退件率</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>达标率</t>
-        </is>
+          <t>上限</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>0.02</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -2114,83 +2091,79 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>达标单数 / 总单数</t>
+          <t>物流因素退件率(小数)</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>头程大表；长期易仓</t>
+          <t>客服数据</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>当月签收，按运输方式分段</t>
+          <t>≤2%</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>K24</t>
+          <t>K21</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>张雨洁</t>
+          <t>吴定佳</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>进口业务</t>
+          <t>C端库存</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>时效</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>达标率</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
+          <t>库存综合</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>达标单数 / 总单数</t>
+          <t>长周期占比(小数) / 平均库龄(天) / 单台库内成本(欧)</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>待定</t>
+          <t>各仓库存表+账单</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>分段标准8月底前定，否则首月NA</t>
+          <t>≤3%/≤120天/≤5欧</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>K25</t>
+          <t>K22</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>张雨洁</t>
+          <t>吴定佳</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2200,7 +2173,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>账单协同-请款</t>
+          <t>请款-C端仓库内</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2224,7 +2197,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>协同雨洁表格</t>
+          <t>10号前，≥90%</t>
         </is>
       </c>
     </row>
@@ -2422,7 +2395,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P44"/>
+  <dimension ref="A1:P43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2911,7 +2884,7 @@
         <v/>
       </c>
       <c r="N10" t="n">
-        <v>15</v>
+        <v>7.5</v>
       </c>
       <c r="O10">
         <f>IF(AND($H10="是",ISNUMBER($M10)),$N10,0)</f>
@@ -2964,7 +2937,7 @@
         <v/>
       </c>
       <c r="N11" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="O11">
         <f>IF(AND($H11="是",ISNUMBER($M11)),$N11,0)</f>
@@ -3017,7 +2990,7 @@
         <v/>
       </c>
       <c r="N12" t="n">
-        <v>25</v>
+        <v>12.5</v>
       </c>
       <c r="O12">
         <f>IF(AND($H12="是",ISNUMBER($M12)),$N12,0)</f>
@@ -3066,7 +3039,7 @@
         <v/>
       </c>
       <c r="N13" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="O13">
         <f>IF(AND($H13="是",ISNUMBER($M13)),$N13,0)</f>
@@ -3080,35 +3053,33 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>K11</t>
+          <t>K23</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>黄婷</t>
+          <t>郑舒漫</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>B端中转</t>
+          <t>特殊发运</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>成本</t>
+          <t>时效</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>成本-计算</t>
-        </is>
-      </c>
-      <c r="F14" t="n">
-        <v>15</v>
-      </c>
+          <t>达标率</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="n"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>欧/台</t>
+          <t>%</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -3117,11 +3088,11 @@
         </is>
       </c>
       <c r="M14">
-        <f>IFERROR(IF($H14&lt;&gt;"是","",IF(OR($I14=0,$I14=""),"",MIN(100,100*$F14/($J14/$I14)))),"")</f>
+        <f>IFERROR(IF($H14&lt;&gt;"是","",IF(OR($J14=0,$J14=""),"",MIN(100,$I14/$J14*100))),"")</f>
         <v/>
       </c>
       <c r="N14" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="O14">
         <f>IF(AND($H14="是",ISNUMBER($M14)),$N14,0)</f>
@@ -3135,17 +3106,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>K12</t>
+          <t>K24</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>黄婷</t>
+          <t>郑舒漫</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>B端中转</t>
+          <t>进口业务</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -3174,7 +3145,7 @@
         <v/>
       </c>
       <c r="N15" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="O15">
         <f>IF(AND($H15="是",ISNUMBER($M15)),$N15,0)</f>
@@ -3188,45 +3159,38 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>K13</t>
+          <t>K25</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>黄婷</t>
+          <t>郑舒漫</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>目的国计划</t>
+          <t>财务</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>缺货率</t>
+          <t>账单协同-请款</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>上限</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
+          <t>请款</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="I16" s="4" t="n"/>
+      <c r="J16" s="4" t="n"/>
       <c r="M16">
-        <f>IFERROR(IF($H16&lt;&gt;"是","",IF($I16="","",IF($I16&lt;=$F16,100,100*$F16/$I16))),"")</f>
+        <f>IFERROR(IF($H16&lt;&gt;"是","",IF(OR($I16="",$J16=""),"",0.5*MAX(0,100-20*$I16)+0.5*MIN(100,$J16/0.9*100))),"")</f>
         <v/>
       </c>
       <c r="N16" t="n">
@@ -3244,7 +3208,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>K14</t>
+          <t>K11</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -3254,25 +3218,25 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>目的国计划</t>
+          <t>B端中转</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>缺货时间</t>
+          <t>成本</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>上限</t>
+          <t>成本-计算</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>天</t>
+          <t>欧/台</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -3281,11 +3245,11 @@
         </is>
       </c>
       <c r="M17">
-        <f>IFERROR(IF($H17&lt;&gt;"是","",IF($I17="","",IF($I17&lt;=$F17,100,100*$F17/$I17))),"")</f>
+        <f>IFERROR(IF($H17&lt;&gt;"是","",IF(OR($I17=0,$I17=""),"",MIN(100,100*$F17/($J17/$I17)))),"")</f>
         <v/>
       </c>
       <c r="N17" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="O17">
         <f>IF(AND($H17="是",ISNUMBER($M17)),$N17,0)</f>
@@ -3299,7 +3263,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>K15</t>
+          <t>K12</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3309,32 +3273,36 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>B端库存</t>
+          <t>B端中转</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>时效</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>库存综合</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr"/>
+          <t>达标率</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="n"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="I18" s="4" t="n"/>
       <c r="M18">
-        <f>IFERROR(IF($H18&lt;&gt;"是","",IF(OR($I18="",$J18="",$K18=""),"",AVERAGE(IF($I18&lt;=0.03,100,100*0.03/$I18),IF($J18&lt;=120,100,100*120/$J18),IF($K18&lt;=5,100,100*5/$K18)))),"")</f>
+        <f>IFERROR(IF($H18&lt;&gt;"是","",IF(OR($J18=0,$J18=""),"",MIN(100,$I18/$J18*100))),"")</f>
         <v/>
       </c>
       <c r="N18" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="O18">
         <f>IF(AND($H18="是",ISNUMBER($M18)),$N18,0)</f>
@@ -3348,7 +3316,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>K16</t>
+          <t>K13</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3358,32 +3326,39 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>财务</t>
+          <t>目的国计划</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>请款-B端仓库内</t>
+          <t>缺货率</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>请款</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr"/>
+          <t>上限</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="J19" s="4" t="n"/>
+      <c r="I19" s="4" t="n"/>
       <c r="M19">
-        <f>IFERROR(IF($H19&lt;&gt;"是","",IF(OR($I19="",$J19=""),"",0.5*MAX(0,100-20*$I19)+0.5*MIN(100,$J19/0.9*100))),"")</f>
+        <f>IFERROR(IF($H19&lt;&gt;"是","",IF($I19="","",IF($I19&lt;=$F19,100,100*$F19/$I19))),"")</f>
         <v/>
       </c>
       <c r="N19" t="n">
-        <v>7.5</v>
+        <v>5</v>
       </c>
       <c r="O19">
         <f>IF(AND($H19="是",ISNUMBER($M19)),$N19,0)</f>
@@ -3397,7 +3372,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>K17</t>
+          <t>K14</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3407,32 +3382,38 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>财务</t>
+          <t>目的国计划</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>请款-海外仓调拨</t>
+          <t>缺货时间</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>请款</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr"/>
+          <t>上限</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>7</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>天</t>
+        </is>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="J20" s="4" t="n"/>
       <c r="M20">
-        <f>IFERROR(IF($H20&lt;&gt;"是","",IF(OR($I20="",$J20=""),"",0.5*MAX(0,100-20*$I20)+0.5*MIN(100,$J20/0.9*100))),"")</f>
+        <f>IFERROR(IF($H20&lt;&gt;"是","",IF($I20="","",IF($I20&lt;=$F20,100,100*$F20/$I20))),"")</f>
         <v/>
       </c>
       <c r="N20" t="n">
-        <v>7.5</v>
+        <v>5</v>
       </c>
       <c r="O20">
         <f>IF(AND($H20="是",ISNUMBER($M20)),$N20,0)</f>
@@ -3446,48 +3427,42 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>K18</t>
+          <t>K15</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>吴定佳</t>
+          <t>黄婷</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>一件代发</t>
+          <t>B端库存</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>成本</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>成本-计算</t>
-        </is>
-      </c>
-      <c r="F21" t="n">
-        <v>15</v>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>欧/台</t>
-        </is>
-      </c>
+          <t>库存综合</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
+      <c r="I21" s="4" t="n"/>
       <c r="M21">
-        <f>IFERROR(IF($H21&lt;&gt;"是","",IF(OR($I21=0,$I21=""),"",MIN(100,100*$F21/($J21/$I21)))),"")</f>
+        <f>IFERROR(IF($H21&lt;&gt;"是","",IF(OR($I21="",$J21="",$K21=""),"",AVERAGE(IF($I21&lt;=0.03,100,100*0.03/$I21),IF($J21&lt;=120,100,100*120/$J21),IF($K21&lt;=5,100,100*5/$K21)))),"")</f>
         <v/>
       </c>
       <c r="N21" t="n">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="O21">
         <f>IF(AND($H21="是",ISNUMBER($M21)),$N21,0)</f>
@@ -3501,46 +3476,42 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>K19</t>
+          <t>K16</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>吴定佳</t>
+          <t>黄婷</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>一件代发</t>
+          <t>财务</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>时效</t>
+          <t>请款-B端仓库内</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>达标率</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="n"/>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
+          <t>请款</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
+      <c r="J22" s="4" t="n"/>
       <c r="M22">
-        <f>IFERROR(IF($H22&lt;&gt;"是","",IF(OR($J22=0,$J22=""),"",MIN(100,$I22/$J22*100))),"")</f>
+        <f>IFERROR(IF($H22&lt;&gt;"是","",IF(OR($I22="",$J22=""),"",0.5*MAX(0,100-20*$I22)+0.5*MIN(100,$J22/0.9*100))),"")</f>
         <v/>
       </c>
       <c r="N22" t="n">
-        <v>16</v>
+        <v>7.5</v>
       </c>
       <c r="O22">
         <f>IF(AND($H22="是",ISNUMBER($M22)),$N22,0)</f>
@@ -3554,49 +3525,42 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>K20</t>
+          <t>K17</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>吴定佳</t>
+          <t>黄婷</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>售后物流</t>
+          <t>财务</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>退件率</t>
+          <t>请款-海外仓调拨</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>上限</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
+          <t>请款</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="I23" s="4" t="n"/>
+      <c r="J23" s="4" t="n"/>
       <c r="M23">
-        <f>IFERROR(IF($H23&lt;&gt;"是","",IF($I23="","",IF($I23&lt;=$F23,100,100*$F23/$I23))),"")</f>
+        <f>IFERROR(IF($H23&lt;&gt;"是","",IF(OR($I23="",$J23=""),"",0.5*MAX(0,100-20*$I23)+0.5*MIN(100,$J23/0.9*100))),"")</f>
         <v/>
       </c>
       <c r="N23" t="n">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="O23">
         <f>IF(AND($H23="是",ISNUMBER($M23)),$N23,0)</f>
@@ -3610,7 +3574,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>K21</t>
+          <t>K18</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3620,32 +3584,38 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>C端库存</t>
+          <t>一件代发</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>成本</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>库存综合</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr"/>
+          <t>成本-计算</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>15</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>欧/台</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="I24" s="4" t="n"/>
       <c r="M24">
-        <f>IFERROR(IF($H24&lt;&gt;"是","",IF(OR($I24="",$J24="",$K24=""),"",AVERAGE(IF($I24&lt;=0.03,100,100*0.03/$I24),IF($J24&lt;=120,100,100*120/$J24),IF($K24&lt;=5,100,100*5/$K24)))),"")</f>
+        <f>IFERROR(IF($H24&lt;&gt;"是","",IF(OR($I24=0,$I24=""),"",MIN(100,100*$F24/($J24/$I24)))),"")</f>
         <v/>
       </c>
       <c r="N24" t="n">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="O24">
         <f>IF(AND($H24="是",ISNUMBER($M24)),$N24,0)</f>
@@ -3659,7 +3629,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>K22</t>
+          <t>K19</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3669,32 +3639,36 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>财务</t>
+          <t>一件代发</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>请款-C端仓库内</t>
+          <t>时效</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>请款</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr"/>
+          <t>达标率</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="n"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
       <c r="H25" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="J25" s="4" t="n"/>
       <c r="M25">
-        <f>IFERROR(IF($H25&lt;&gt;"是","",IF(OR($I25="",$J25=""),"",0.5*MAX(0,100-20*$I25)+0.5*MIN(100,$J25/0.9*100))),"")</f>
+        <f>IFERROR(IF($H25&lt;&gt;"是","",IF(OR($J25=0,$J25=""),"",MIN(100,$I25/$J25*100))),"")</f>
         <v/>
       </c>
       <c r="N25" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="O25">
         <f>IF(AND($H25="是",ISNUMBER($M25)),$N25,0)</f>
@@ -3708,30 +3682,32 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>K23</t>
+          <t>K20</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>张雨洁</t>
+          <t>吴定佳</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>特殊发运</t>
+          <t>售后物流</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>时效</t>
+          <t>退件率</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>达标率</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="n"/>
+          <t>上限</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="n">
+        <v>0.02</v>
+      </c>
       <c r="G26" t="inlineStr">
         <is>
           <t>%</t>
@@ -3742,12 +3718,13 @@
           <t>是</t>
         </is>
       </c>
+      <c r="I26" s="4" t="n"/>
       <c r="M26">
-        <f>IFERROR(IF($H26&lt;&gt;"是","",IF(OR($J26=0,$J26=""),"",MIN(100,$I26/$J26*100))),"")</f>
+        <f>IFERROR(IF($H26&lt;&gt;"是","",IF($I26="","",IF($I26&lt;=$F26,100,100*$F26/$I26))),"")</f>
         <v/>
       </c>
       <c r="N26" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="O26">
         <f>IF(AND($H26="是",ISNUMBER($M26)),$N26,0)</f>
@@ -3761,46 +3738,42 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>K24</t>
+          <t>K21</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>张雨洁</t>
+          <t>吴定佳</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>进口业务</t>
+          <t>C端库存</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>时效</t>
+          <t>综合</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>达标率</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="n"/>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
+          <t>库存综合</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
+      <c r="I27" s="4" t="n"/>
       <c r="M27">
-        <f>IFERROR(IF($H27&lt;&gt;"是","",IF(OR($J27=0,$J27=""),"",MIN(100,$I27/$J27*100))),"")</f>
+        <f>IFERROR(IF($H27&lt;&gt;"是","",IF(OR($I27="",$J27="",$K27=""),"",AVERAGE(IF($I27&lt;=0.03,100,100*0.03/$I27),IF($J27&lt;=120,100,100*120/$J27),IF($K27&lt;=5,100,100*5/$K27)))),"")</f>
         <v/>
       </c>
       <c r="N27" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="O27">
         <f>IF(AND($H27="是",ISNUMBER($M27)),$N27,0)</f>
@@ -3814,12 +3787,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>K25</t>
+          <t>K22</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>张雨洁</t>
+          <t>吴定佳</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -3829,7 +3802,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>账单协同-请款</t>
+          <t>请款-C端仓库内</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -3996,7 +3969,7 @@
         </is>
       </c>
       <c r="M31">
-        <f>IFERROR(IF($H31&lt;&gt;"是","",IFERROR(AVERAGE($M$9,$M$13,$M$19,$M$20,$M$25,$M$28),"")),"")</f>
+        <f>IFERROR(IF($H31&lt;&gt;"是","",IFERROR(AVERAGE($M$9,$M$13,$M$22,$M$23,$M$28,$M$16),"")),"")</f>
         <v/>
       </c>
       <c r="N31" t="n">
@@ -4180,11 +4153,11 @@
         </is>
       </c>
       <c r="B40">
-        <f>SUM($O$10:$O$13)</f>
+        <f>SUM($O$10:$O$16)</f>
         <v/>
       </c>
       <c r="C40">
-        <f>SUM($P$10:$P$13)</f>
+        <f>SUM($P$10:$P$16)</f>
         <v/>
       </c>
       <c r="D40">
@@ -4207,11 +4180,11 @@
         </is>
       </c>
       <c r="B41">
-        <f>SUM($O$14:$O$20)</f>
+        <f>SUM($O$17:$O$23)</f>
         <v/>
       </c>
       <c r="C41">
-        <f>SUM($P$14:$P$20)</f>
+        <f>SUM($P$17:$P$23)</f>
         <v/>
       </c>
       <c r="D41">
@@ -4234,11 +4207,11 @@
         </is>
       </c>
       <c r="B42">
-        <f>SUM($O$21:$O$25)</f>
+        <f>SUM($O$24:$O$28)</f>
         <v/>
       </c>
       <c r="C42">
-        <f>SUM($P$21:$P$25)</f>
+        <f>SUM($P$24:$P$28)</f>
         <v/>
       </c>
       <c r="D42">
@@ -4257,15 +4230,15 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>张雨洁</t>
+          <t>金炜铮</t>
         </is>
       </c>
       <c r="B43">
-        <f>SUM($O$26:$O$28)</f>
+        <f>SUM($O$29:$O$32)</f>
         <v/>
       </c>
       <c r="C43">
-        <f>SUM($P$26:$P$28)</f>
+        <f>SUM($P$29:$P$32)</f>
         <v/>
       </c>
       <c r="D43">
@@ -4278,33 +4251,6 @@
       </c>
       <c r="F43">
         <f>IFERROR((C43+IF(ISNUMBER(D43),D43*30,0))/(B43+IF(ISNUMBER(D43),30,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>金炜铮</t>
-        </is>
-      </c>
-      <c r="B44">
-        <f>SUM($O$29:$O$32)</f>
-        <v/>
-      </c>
-      <c r="C44">
-        <f>SUM($P$29:$P$32)</f>
-        <v/>
-      </c>
-      <c r="D44">
-        <f>IFERROR(AVERAGEIFS(任务块!$E:$E,任务块!$B:$B,$A44,任务块!$A:$A,$B$1),"")</f>
-        <v/>
-      </c>
-      <c r="E44" s="5">
-        <f>B44/70</f>
-        <v/>
-      </c>
-      <c r="F44">
-        <f>IFERROR((C44+IF(ISNUMBER(D44),D44*30,0))/(B44+IF(ISNUMBER(D44),30,0)),"")</f>
         <v/>
       </c>
     </row>
@@ -4324,7 +4270,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4486,17 +4432,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>张雨洁</t>
+          <t>郑舒漫</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>进口时效分段标准整理</t>
+          <t>雨洁工作交接验收（9/7）</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>分段标准表（无现成标准则注明NA）</t>
+          <t>交接文档+实单演练，特殊发运/进口/单据可独立跑</t>
         </is>
       </c>
     </row>
@@ -4508,15 +4454,37 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>郑舒漫</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>特殊发运时效分段标准</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>分段标准表（无现成标准则注明NA）</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>金炜铮</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>绩效体系首月跑通+复盘</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>首月记分卡+看板产出+修订清单</t>
         </is>

</xml_diff>